<commit_message>
Amend preregistration to ten-card draw
</commit_message>
<xml_diff>
--- a/preregistration/BackspaceGate.xlsx
+++ b/preregistration/BackspaceGate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taylor/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE731F75-5A99-2345-8803-32772F884D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED5C0AA-20C0-B348-B995-E2994CCED5C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1580" yWindow="700" windowWidth="21140" windowHeight="16680" activeTab="2" xr2:uid="{1DF52C0B-E756-0F48-A2FB-F0CCDE2B9253}"/>
   </bookViews>
@@ -283,48 +283,27 @@
     <t>Hypothesis</t>
   </si>
   <si>
-    <t>Transcript-mediated inspection will recover the concealed 8-word sequence exactly.</t>
-  </si>
-  <si>
-    <t>The frozen recovery is independent of the concealed target; an exact ordered match occurs by chance.</t>
-  </si>
-  <si>
     <t>Independent variable</t>
   </si>
   <si>
-    <t>Concealed 8-word target drawn without replacement from a human-generated pool of 100 unique words.</t>
-  </si>
-  <si>
     <t>Dependent variable</t>
   </si>
   <si>
-    <t>Correct ordered word positions / 8; exact-string match (0/1).</t>
-  </si>
-  <si>
     <t>Statistics</t>
   </si>
   <si>
-    <t>One-sided exact Spearman rank correlation; alpha = .05.</t>
-  </si>
-  <si>
     <t>Spearman (1904); Best &amp; Roberts (1975); R Core Team (2026); Wasserstein &amp; Lazar (2016)</t>
   </si>
   <si>
     <t>Math</t>
   </si>
   <si>
-    <t>P(100,8) = 100! / 92! = 7,503,063,898,176,000; Pr(exact ordered match | H0) = 1 / P(100,8) = 1.332788862751256E-16; Pr(rho = 1 | correct identities, random order) = 1 / 8! = 2.480158730158730E-5.</t>
-  </si>
-  <si>
     <t>Abramson &amp; North (2020); Best &amp; Roberts (1975); R Core Team (2026)</t>
   </si>
   <si>
     <t>Prediction</t>
   </si>
   <si>
-    <t>8/8 correct; ordered-word accuracy = 100%; exact-string match = 1; rho = 1.000.</t>
-  </si>
-  <si>
     <t>Spearman (1904)</t>
   </si>
   <si>
@@ -347,6 +326,27 @@
   </si>
   <si>
     <t>Wasserstein, R. L., &amp; Lazar, N. A. (2016). The ASA's statement on p-values: Context, process, and purpose. The American Statistician, 70(2), 129-133. https://doi.org/10.1080/00031305.2016.1154108</t>
+  </si>
+  <si>
+    <t>Transcript-mediated inspection will recover the concealed ordered 10-card sequence exactly.</t>
+  </si>
+  <si>
+    <t>The frozen recovery is independent of the concealed card order; an exact ordered match occurs by chance.</t>
+  </si>
+  <si>
+    <t>Concealed ordered 10-card sequence drawn without replacement from a shuffled standard 52-card deck (no jokers).</t>
+  </si>
+  <si>
+    <t>Correct ordered card positions / 10; exact-sequence match (0/1).</t>
+  </si>
+  <si>
+    <t>P(52,10) = 52! / 42! = 57,407,703,889,536,000; Pr(exact ordered match | H0) = 1 / P(52,10) = 1.741926487643891E-17; Pr(rho = 1 | correct identities, random order) = 1 / 10! = 2.755731922398589E-7.</t>
+  </si>
+  <si>
+    <t>10/10 correct; ordered-card accuracy = 100%; exact-sequence match = 1; rho = 1.000.</t>
+  </si>
+  <si>
+    <t>Primary: exact ordered-sequence permutation test; secondary: Spearman rho; alpha = .05.</t>
   </si>
 </sst>
 </file>
@@ -1038,37 +1038,37 @@
   <sheetData>
     <row r="1" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="306" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="372" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="306" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="306" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="306" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="356" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1102,68 +1102,68 @@
         <v>79</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>